<commit_message>
Axi Academy quiz bank: apply the fact-check, bookmarks, final PDF and Excel
- Fact-check found no wrong keys; fixed its 24 findings (one date, five
  arguable options, two compliance wordings, fourteen giveaways between
  questions in the same set, two wording slips) plus one more giveaway
  found while checking the layout.
- PDF: correct right-to-left bookmarks for every course and lesson
  (tool/bookmarks.py), clickable contents, document title.
- README: review results, decisions, build steps.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9b7SosS81gsG93Ye2rtJ2
</commit_message>
<xml_diff>
--- a/axi-academy/quizzes/AxiAcademy_QuestionBank.xlsx
+++ b/axi-academy/quizzes/AxiAcademy_QuestionBank.xlsx
@@ -837,7 +837,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>كم دولاراً أسترالياً استلم جون عندما أعاد تحويل الـ 700 دولار أمريكي؟</t>
+          <t>كم دولاراً أسترالياً استلم جون عندما أعاد تحويل دولاراته الأمريكية؟</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1002,7 +1002,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>لو انخفضت قيمة الدولار الأمريكي مقابل الدولار الأسترالي بدلاً من ارتفاعها، فماذا كان سيحدث عند إعادة التحويل؟</t>
+          <t>إذا انخفضت قيمة الدولار الأمريكي مقابل الدولار الأسترالي بين التحويلين، فماذا يحدث عند إعادة التحويل؟</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1772,27 +1772,27 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>ما زوج العملات في مثال جون الذي خطّط للسفر من أستراليا إلى أمريكا؟</t>
+          <t>لماذا كان زوج AUD/USD هو الزوج المعني في مثال جون؟</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>الدولار الأمريكي مقابل الين الياباني (USD/JPY)</t>
+          <t>لأن الوسيط لا يعرض أي زوج غيره</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>الدولار الأسترالي مقابل الدولار الأمريكي (AUD/USD)</t>
+          <t>لأنه أراد تحويل دولاراته الأسترالية إلى دولارات أمريكية للسفر إلى أمريكا</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>اليورو مقابل الدولار الأمريكي (EUR/USD)</t>
+          <t>لأنه أكثر أزواج العملات تداولاً في العالم</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>الجنيه الإسترليني مقابل الدولار الأمريكي (GBP/USD)</t>
+          <t>لأن الدولار الأسترالي يساوي الدولار الأمريكي دائماً</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>الدولار الأسترالي مقابل الدولار الأمريكي (AUD/USD)</t>
+          <t>لأنه أراد تحويل دولاراته الأسترالية إلى دولارات أمريكية للسفر إلى أمريكا</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>إذا قوي الدولار الأمريكي أمام الدولار الأسترالي، فماذا يحدث غالباً لسعر AUD/USD؟</t>
+          <t>إذا قوي الدولار الأمريكي أمام الدولار الأسترالي، فماذا يحدث لسعر AUD/USD؟</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -4302,27 +4302,27 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>في صفقة شراء، أين يوضع هدف جني الأرباح؟</t>
+          <t>حسب درس المصطلحات، أي أدوات التداول تتطلب عادةً هامشاً أكبر؟</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>فوق سعر الدخول</t>
+          <t>السلع</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>عند مستوى وقف الخسارة</t>
+          <t>لا توجد أداة تتطلب هامشاً</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>عند سعر الدخول نفسه</t>
+          <t>كل الأدوات تتطلب الهامش نفسه</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>تحت سعر الدخول</t>
+          <t>الفوركس</t>
         </is>
       </c>
       <c r="J70" s="5" t="inlineStr">
@@ -4332,7 +4332,7 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>فوق سعر الدخول</t>
+          <t>السلع</t>
         </is>
       </c>
     </row>
@@ -4417,7 +4417,7 @@
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>لحمايتك من خسارة أكثر مما أودعت</t>
+          <t>لإيقاف خسائرك عندما لا يعود هامشك كافياً لإبقاء الصفقة مفتوحة</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>لحمايتك من خسارة أكثر مما أودعت</t>
+          <t>لإيقاف خسائرك عندما لا يعود هامشك كافياً لإبقاء الصفقة مفتوحة</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>رفع الرافعة المالية</t>
+          <t>زيادة حجم الصفقة</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -4977,7 +4977,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>أن نوع الرسم لا يؤثر في الأسعار</t>
+          <t>أن كل المتداولين يفسّرون الرسم البياني بالطريقة نفسها</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -5017,27 +5017,27 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>ما العلاقة المعتادة بين سعر العرض (Ask) وسعر الطلب (Bid)؟</t>
+          <t>قال متداول: «ربحت 100 نقطة في هذه الصفقة». ماذا يعني ذلك؟</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>لا علاقة بينهما</t>
+          <t>أن السعر تحرّك 100 خانة عشرية</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>سعر الطلب أعلى من سعر العرض</t>
+          <t>أنه ربح 100 دولار بالضبط مهما كان حجم صفقته</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
         <is>
-          <t>سعر العرض أعلى من سعر الطلب</t>
+          <t>أن السعر تحرّك لصالحه بمقدار 100 نقطة</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>السعران متساويان دائماً</t>
+          <t>أنه فتح 100 صفقة رابحة</t>
         </is>
       </c>
       <c r="J83" s="5" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>سعر العرض أعلى من سعر الطلب</t>
+          <t>أن السعر تحرّك لصالحه بمقدار 100 نقطة</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>فتحت صفقة شراء عند سعر العرض (Ask). بأي سعر تُغلق هذه الصفقة؟</t>
+          <t>فتحت صفقة شراء. بأي سعر تُغلق هذه الصفقة؟</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -7437,7 +7437,7 @@
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>اشتريت سهماً عند 150 دولاراً ووضعت جني الأرباح عند 160 دولاراً، ووصل السعر إلى الهدف. كم ربحت في السهم الواحد؟</t>
+          <t>اشتريت سهماً عند 200 دولار ووضعت جني الأرباح عند 215 دولاراً، ووصل السعر إلى الهدف. كم ربحت في السهم الواحد؟</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -7447,17 +7447,17 @@
       </c>
       <c r="G127" s="4" t="inlineStr">
         <is>
-          <t>10 دولارات</t>
+          <t>15 دولاراً</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>150 دولاراً</t>
+          <t>200 دولار</t>
         </is>
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>160 دولاراً</t>
+          <t>215 دولاراً</t>
         </is>
       </c>
       <c r="J127" s="5" t="inlineStr">
@@ -7467,7 +7467,7 @@
       </c>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>10 دولارات</t>
+          <t>15 دولاراً</t>
         </is>
       </c>
     </row>
@@ -8057,7 +8057,7 @@
       </c>
       <c r="H138" s="4" t="inlineStr">
         <is>
-          <t>يمنعك من خسارة أكثر مما خطّطت له أو مما تستطيع تحمّله</t>
+          <t>يحدّ من خسارتك عند مستوى تحدّده مسبقاً</t>
         </is>
       </c>
       <c r="I138" s="2" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="K138" s="2" t="inlineStr">
         <is>
-          <t>يمنعك من خسارة أكثر مما خطّطت له أو مما تستطيع تحمّله</t>
+          <t>يحدّ من خسارتك عند مستوى تحدّده مسبقاً</t>
         </is>
       </c>
     </row>
@@ -8207,29 +8207,29 @@
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>في صفقة شراء، أين يوضع وقف الخسارة عادةً؟</t>
+          <t>في صفقة بيع (Sell)، أين يوضع وقف الخسارة عادةً؟</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
+          <t>تحت سعر الدخول</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>عند هدف جني الأرباح</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>عند سعر الدخول نفسه</t>
+        </is>
+      </c>
+      <c r="I141" s="4" t="inlineStr">
+        <is>
           <t>فوق سعر الدخول</t>
         </is>
       </c>
-      <c r="G141" s="2" t="inlineStr">
-        <is>
-          <t>عند هدف جني الأرباح</t>
-        </is>
-      </c>
-      <c r="H141" s="2" t="inlineStr">
-        <is>
-          <t>عند سعر الدخول نفسه</t>
-        </is>
-      </c>
-      <c r="I141" s="4" t="inlineStr">
-        <is>
-          <t>تحت سعر الدخول</t>
-        </is>
-      </c>
       <c r="J141" s="5" t="inlineStr">
         <is>
           <t>د</t>
@@ -8237,7 +8237,7 @@
       </c>
       <c r="K141" s="2" t="inlineStr">
         <is>
-          <t>تحت سعر الدخول</t>
+          <t>فوق سعر الدخول</t>
         </is>
       </c>
     </row>
@@ -8927,7 +8927,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>عند منتصف الليل بتوقيت بغداد</t>
+          <t>عند الساعة 12:00 ظهراً بتوقيت بغداد</t>
         </is>
       </c>
       <c r="G154" s="4" t="inlineStr">
@@ -10022,7 +10022,7 @@
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>تريد فتح صفقة بحجم عقد واحد من EUR/USD (أي 100,000 يورو) برافعة 1 إلى 200، وسعر اليورو يساوي 1 دولار. كم الهامش المطلوب؟</t>
+          <t>تريد فتح صفقة بحجم عقد واحد من EUR/USD برافعة 1 إلى 200، وسعر اليورو يساوي 1 دولار. كم الهامش المطلوب؟</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
@@ -10297,7 +10297,7 @@
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>تتداول زوج GBP/USD. بأي عملة يُحسب الهامش؟</t>
+          <t>حسب الدرس، بأي عملة يُحسب الهامش عند تداول زوج GBP/USD؟</t>
         </is>
       </c>
       <c r="F179" s="4" t="inlineStr">
@@ -10737,7 +10737,7 @@
       </c>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>اشتريت EUR/USD عند 1.1000، ووقف الخسارة عند 1.0950، وجني الأرباح عند 1.1100. ماذا يحدث إذا هبط السعر إلى 1.0950؟</t>
+          <t>اشتريت EUR/USD ووضعت وقف الخسارة على بُعد 50 نقطة من سعر الدخول. ماذا يحدث إذا تحرّك السعر 50 نقطة ضدك؟</t>
         </is>
       </c>
       <c r="F187" s="4" t="inlineStr">
@@ -10747,12 +10747,12 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>تبقى مفتوحة حتى يصل السعر إلى 1.1100</t>
+          <t>تبقى مفتوحة حتى تغلقها يدوياً</t>
         </is>
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
-          <t>تُغلق الصفقة تلقائياً بربح 100 نقطة</t>
+          <t>تُغلق الصفقة تلقائياً بربح 50 نقطة</t>
         </is>
       </c>
       <c r="I187" s="2" t="inlineStr">
@@ -10792,37 +10792,37 @@
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>فتحت صفقة بيع عند 1.2000. أين يوضع وقف الخسارة عادةً؟</t>
+          <t>بعت زوج عملات عند 1.3000 ووضعت وقف الخسارة عند 1.3030. كم نقطة تخاطر بها؟</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>لا يُستخدم وقف الخسارة في صفقات البيع</t>
-        </is>
-      </c>
-      <c r="G188" s="2" t="inlineStr">
-        <is>
-          <t>تحت سعر الدخول، مثل 1.1950</t>
+          <t>3 نقاط</t>
+        </is>
+      </c>
+      <c r="G188" s="4" t="inlineStr">
+        <is>
+          <t>30 نقطة</t>
         </is>
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>عند سعر الدخول نفسه</t>
-        </is>
-      </c>
-      <c r="I188" s="4" t="inlineStr">
-        <is>
-          <t>فوق سعر الدخول، مثل 1.2050</t>
+          <t>300 نقطة</t>
+        </is>
+      </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>3,000 نقطة</t>
         </is>
       </c>
       <c r="J188" s="5" t="inlineStr">
         <is>
-          <t>د</t>
+          <t>ب</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr">
         <is>
-          <t>فوق سعر الدخول، مثل 1.2050</t>
+          <t>30 نقطة</t>
         </is>
       </c>
     </row>
@@ -10905,29 +10905,29 @@
           <t>وضعت جني الأرباح ووقف الخسارة لصفقة شراء. أي ترتيب صحيح للمستويات من الأدنى إلى الأعلى؟</t>
         </is>
       </c>
-      <c r="F190" s="4" t="inlineStr">
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>وقف الخسارة، ثم جني الأرباح، ثم سعر الدخول</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>جني الأرباح، ثم سعر الدخول، ثم وقف الخسارة</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>سعر الدخول، ثم وقف الخسارة، ثم جني الأرباح</t>
+        </is>
+      </c>
+      <c r="I190" s="4" t="inlineStr">
         <is>
           <t>وقف الخسارة، ثم سعر الدخول، ثم جني الأرباح</t>
         </is>
       </c>
-      <c r="G190" s="2" t="inlineStr">
-        <is>
-          <t>جني الأرباح، ثم سعر الدخول، ثم وقف الخسارة</t>
-        </is>
-      </c>
-      <c r="H190" s="2" t="inlineStr">
-        <is>
-          <t>سعر الدخول، ثم وقف الخسارة، ثم جني الأرباح</t>
-        </is>
-      </c>
-      <c r="I190" s="2" t="inlineStr">
-        <is>
-          <t>وقف الخسارة، ثم جني الأرباح، ثم سعر الدخول</t>
-        </is>
-      </c>
       <c r="J190" s="5" t="inlineStr">
         <is>
-          <t>أ</t>
+          <t>د</t>
         </is>
       </c>
       <c r="K190" s="2" t="inlineStr">
@@ -10960,29 +10960,29 @@
           <t>السعر الحالي 1.1050، وتريد الشراء عند 1.1000 لأنك تتوقع ارتداد السعر من هذا المستوى. أي أمر تستخدم؟</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr">
+      <c r="F191" s="4" t="inlineStr">
+        <is>
+          <t>أمر الشراء المحدد (Buy Limit)</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>أمر الشراء الموقوف (Buy Stop)</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>أمر البيع المحدد (Sell Limit)</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
         <is>
           <t>أمر البيع الموقوف (Sell Stop)</t>
         </is>
       </c>
-      <c r="G191" s="2" t="inlineStr">
-        <is>
-          <t>أمر البيع المحدد (Sell Limit)</t>
-        </is>
-      </c>
-      <c r="H191" s="2" t="inlineStr">
-        <is>
-          <t>أمر الشراء الموقوف (Buy Stop)</t>
-        </is>
-      </c>
-      <c r="I191" s="4" t="inlineStr">
-        <is>
-          <t>أمر الشراء المحدد (Buy Limit)</t>
-        </is>
-      </c>
       <c r="J191" s="5" t="inlineStr">
         <is>
-          <t>د</t>
+          <t>أ</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr">
@@ -11015,29 +11015,29 @@
           <t>السعر الحالي 1.1050، وتريد الشراء عند 1.1100 إذا اخترق السعر هذا المستوى صعوداً. أي أمر تستخدم؟</t>
         </is>
       </c>
-      <c r="F192" s="4" t="inlineStr">
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>أمر البيع الفوري (Sell Market)</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>أمر البيع الموقوف (Sell Stop)</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>أمر الشراء المحدد (Buy Limit)</t>
+        </is>
+      </c>
+      <c r="I192" s="4" t="inlineStr">
         <is>
           <t>أمر الشراء الموقوف (Buy Stop)</t>
         </is>
       </c>
-      <c r="G192" s="2" t="inlineStr">
-        <is>
-          <t>أمر البيع الموقوف (Sell Stop)</t>
-        </is>
-      </c>
-      <c r="H192" s="2" t="inlineStr">
-        <is>
-          <t>أمر البيع الفوري (Sell Market)</t>
-        </is>
-      </c>
-      <c r="I192" s="2" t="inlineStr">
-        <is>
-          <t>أمر الشراء المحدد (Buy Limit)</t>
-        </is>
-      </c>
       <c r="J192" s="5" t="inlineStr">
         <is>
-          <t>أ</t>
+          <t>د</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11070,29 +11070,29 @@
           <t>السعر الحالي 1.1050، وتريد البيع عند 1.1100 لأنك تتوقع أن يرتد السعر من مقاومة. أي أمر تستخدم؟</t>
         </is>
       </c>
-      <c r="F193" s="2" t="inlineStr">
+      <c r="F193" s="4" t="inlineStr">
+        <is>
+          <t>أمر البيع المحدد (Sell Limit)</t>
+        </is>
+      </c>
+      <c r="G193" s="2" t="inlineStr">
+        <is>
+          <t>أمر الشراء الموقوف (Buy Stop)</t>
+        </is>
+      </c>
+      <c r="H193" s="2" t="inlineStr">
         <is>
           <t>أمر الشراء المحدد (Buy Limit)</t>
         </is>
       </c>
-      <c r="G193" s="2" t="inlineStr">
-        <is>
-          <t>أمر الشراء الموقوف (Buy Stop)</t>
-        </is>
-      </c>
-      <c r="H193" s="2" t="inlineStr">
+      <c r="I193" s="2" t="inlineStr">
         <is>
           <t>أمر البيع الموقوف (Sell Stop)</t>
         </is>
       </c>
-      <c r="I193" s="4" t="inlineStr">
-        <is>
-          <t>أمر البيع المحدد (Sell Limit)</t>
-        </is>
-      </c>
       <c r="J193" s="5" t="inlineStr">
         <is>
-          <t>د</t>
+          <t>أ</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
@@ -11130,24 +11130,24 @@
           <t>أمر البيع المحدد (Sell Limit)</t>
         </is>
       </c>
-      <c r="G194" s="4" t="inlineStr">
+      <c r="G194" s="2" t="inlineStr">
+        <is>
+          <t>أمر البيع الفوري (Sell Market)</t>
+        </is>
+      </c>
+      <c r="H194" s="4" t="inlineStr">
         <is>
           <t>أمر البيع الموقوف (Sell Stop)</t>
         </is>
       </c>
-      <c r="H194" s="2" t="inlineStr">
+      <c r="I194" s="2" t="inlineStr">
         <is>
           <t>أمر الشراء المحدد (Buy Limit)</t>
         </is>
       </c>
-      <c r="I194" s="2" t="inlineStr">
-        <is>
-          <t>أمر البيع الفوري (Sell Market)</t>
-        </is>
-      </c>
       <c r="J194" s="5" t="inlineStr">
         <is>
-          <t>ب</t>
+          <t>ج</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11180,29 +11180,29 @@
           <t>ماذا يعني أمر الشراء الفوري (Buy Market)؟</t>
         </is>
       </c>
-      <c r="F195" s="4" t="inlineStr">
+      <c r="F195" s="2" t="inlineStr">
+        <is>
+          <t>إغلاق جميع الصفقات المفتوحة</t>
+        </is>
+      </c>
+      <c r="G195" s="2" t="inlineStr">
+        <is>
+          <t>تأجيل الصفقة إلى اليوم التالي</t>
+        </is>
+      </c>
+      <c r="H195" s="2" t="inlineStr">
+        <is>
+          <t>فتح الصفقة عند سعر تحدده في المستقبل</t>
+        </is>
+      </c>
+      <c r="I195" s="4" t="inlineStr">
         <is>
           <t>فتح الصفقة عند السعر الحالي للسوق</t>
         </is>
       </c>
-      <c r="G195" s="2" t="inlineStr">
-        <is>
-          <t>إغلاق جميع الصفقات المفتوحة</t>
-        </is>
-      </c>
-      <c r="H195" s="2" t="inlineStr">
-        <is>
-          <t>فتح الصفقة عند سعر تحدده في المستقبل</t>
-        </is>
-      </c>
-      <c r="I195" s="2" t="inlineStr">
-        <is>
-          <t>تأجيل الصفقة إلى اليوم التالي</t>
-        </is>
-      </c>
       <c r="J195" s="5" t="inlineStr">
         <is>
-          <t>أ</t>
+          <t>د</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11235,21 +11235,21 @@
           <t>ما الذي تتيحه إدارة الأوامر المتقدمة في ميتا تريدر؟</t>
         </is>
       </c>
-      <c r="F196" s="2" t="inlineStr">
+      <c r="F196" s="4" t="inlineStr">
+        <is>
+          <t>تتبّع جميع صفقاتك المفتوحة والمعلّقة والمغلقة</t>
+        </is>
+      </c>
+      <c r="G196" s="2" t="inlineStr">
         <is>
           <t>إلغاء الفوارق السعرية</t>
         </is>
       </c>
-      <c r="G196" s="2" t="inlineStr">
+      <c r="H196" s="2" t="inlineStr">
         <is>
           <t>منع أي خسارة في الحساب</t>
         </is>
       </c>
-      <c r="H196" s="4" t="inlineStr">
-        <is>
-          <t>تتبّع جميع صفقاتك المفتوحة والمعلّقة والمغلقة</t>
-        </is>
-      </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
           <t>تحديد أسعار السوق بنفسك</t>
@@ -11257,7 +11257,7 @@
       </c>
       <c r="J196" s="5" t="inlineStr">
         <is>
-          <t>ج</t>
+          <t>أ</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -12552,7 +12552,7 @@
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>ماذا تفعل إذا لم تستوفِ الفرصة شروط قائمة التحقق الخاصة بك؟</t>
+          <t>ماذا تفعل إذا لم تستوفِ الفرصة شروطك؟</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="E223" s="2" t="inlineStr">
         <is>
-          <t>هل يجب أن تطبّق مستوى المخاطرة نفسه على كل صفقة؟</t>
+          <t>حسب الدرس، هل يجب أن تطبّق مستوى المخاطرة نفسه على كل صفقة؟</t>
         </is>
       </c>
       <c r="F223" s="2" t="inlineStr">
@@ -12937,7 +12937,7 @@
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>متى يمكنك رفع المخاطرة إلى 1% أو 1.5%؟</t>
+          <t>متى يمكنك رفع نسبة المخاطرة فوق مستوى البداية؟</t>
         </is>
       </c>
       <c r="F227" s="2" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="E276" s="2" t="inlineStr">
         <is>
-          <t>أي العبارتين تصف الفرق بين التحليلين بدقة؟</t>
+          <t>أي العبارات التالية تصف الفرق بين التحليلين بدقة؟</t>
         </is>
       </c>
       <c r="F276" s="2" t="inlineStr">
@@ -17502,7 +17502,7 @@
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
-          <t>بهامش 5%، ماذا تعني حركة عكسية في السعر بنسبة 5%؟</t>
+          <t>بهامش 20%، ماذا تعني حركة عكسية في السعر بنسبة 20%؟</t>
         </is>
       </c>
       <c r="F310" s="2" t="inlineStr">
@@ -17522,7 +17522,7 @@
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>خسارة 5% من الهامش فقط</t>
+          <t>خسارة 20% من الهامش فقط</t>
         </is>
       </c>
       <c r="J310" s="5" t="inlineStr">
@@ -18547,7 +18547,7 @@
       </c>
       <c r="E329" s="2" t="inlineStr">
         <is>
-          <t>إذا كان اللوت 100 أونصة وتحرّك سعر الأونصة دولاراً واحداً، فكم تقريباً الربح أو الخسارة على لوت كامل؟</t>
+          <t>تحرّك سعر الأونصة دولاراً واحداً. كم تقريباً الربح أو الخسارة على لوت كامل عند كثير من الوسطاء؟</t>
         </is>
       </c>
       <c r="F329" s="2" t="inlineStr">
@@ -18712,7 +18712,7 @@
       </c>
       <c r="E332" s="2" t="inlineStr">
         <is>
-          <t>ما التوقيت الثابت للعراق طوال السنة؟</t>
+          <t>ما توقيت العراق بالنسبة إلى غرينتش؟</t>
         </is>
       </c>
       <c r="F332" s="2" t="inlineStr">
@@ -21407,7 +21407,7 @@
       </c>
       <c r="E381" s="2" t="inlineStr">
         <is>
-          <t>منذ أي عام لا يطبّق العراق التوقيت الصيفي؟</t>
+          <t>بعد أي عام توقّف العراق عن تطبيق التوقيت الصيفي؟</t>
         </is>
       </c>
       <c r="F381" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Quiz bank: general lesson 1 questions with worked conversion problems
At the client's request, lesson 1 no longer refers to the story
character. It asks about forex in general, and the story is replaced by
four conversion problems whose wrong options are typical mistakes.
PDF and Excel rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9b7SosS81gsG93Ye2rtJ2
</commit_message>
<xml_diff>
--- a/axi-academy/quizzes/AxiAcademy_QuestionBank.xlsx
+++ b/axi-academy/quizzes/AxiAcademy_QuestionBank.xlsx
@@ -562,32 +562,32 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>ما المقصود بكلمة «الفوركس»؟</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>اختصار لبورصة السلع والمعادن</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
+          <t>ما المقصود بمصطلح «الفوركس»؟</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>اختصار لسوق الصرف الأجنبي</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>اسم لبورصة السلع والمعادن العالمية</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>اسم لسوق الأسهم العالمية</t>
+          <t>اختصار لسوق الأسهم الأجنبية</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>اسم لسوق السندات الحكومية</t>
+          <t>اسم لنظام التحويلات المصرفية الدولية</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>ب</t>
+          <t>أ</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -617,22 +617,22 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>ما الوظيفة الأساسية لسوق الفوركس كما شرحها الدرس؟</t>
+          <t>ما الوظيفة الأساسية لسوق الفوركس؟</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>إقراض الأموال بفائدة ثابتة</t>
+          <t>تخزين احتياطيات الدول من العملات الأجنبية</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>بيع أسهم الشركات وشراؤها</t>
+          <t>تحديد سعر صرف ثابت لكل عملة مقابل الدولار</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>تخزين الذهب والمعادن الثمينة</t>
+          <t>إقراض الحكومات بالعملات الأجنبية</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
@@ -672,17 +672,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>لماذا تتغير قيمة الصرف بين العملات باستمرار؟</t>
+          <t>لماذا تتغير أسعار الصرف بين العملات باستمرار؟</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>لأن مكاتب الصرافة تحدّدها بشكل عشوائي</t>
+          <t>لأن مكاتب الصرافة تغيّرها لتحقيق أرباحها</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>لأن قيمة العملات تتغير مرة واحدة فقط كل سنة</t>
+          <t>لأن قيمة كل عملة مربوطة بسعر ثابت للذهب</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>لأن حركة السفر بين الدول تتوقف أحياناً</t>
+          <t>لأن البنوك المركزية تعيد تحديدها كل ساعة بقرار رسمي</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -727,37 +727,37 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>في مثال الدرس، كم دولاراً أمريكياً حصل جون مقابل 1,000 دولار أسترالي؟</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>700 دولار أمريكي</t>
+          <t>ماذا يعني أن عملة ما «قويت» مقابل عملة أخرى؟</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>أن الكمية المطبوعة منها زادت</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>900 دولار أمريكي</t>
+          <t>أن سعر صرفها أصبح ثابتاً لا يتغير</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>1,000 دولار أمريكي</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>1,100 دولار أمريكي</t>
+          <t>أن سعر الفائدة عليها ارتفع</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>أن الوحدة الواحدة منها أصبحت تساوي كمية أكبر من العملة الأخرى</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>أ</t>
+          <t>د</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>700 دولار أمريكي</t>
+          <t>أن الوحدة الواحدة منها أصبحت تساوي كمية أكبر من العملة الأخرى</t>
         </is>
       </c>
     </row>
@@ -782,37 +782,37 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>لماذا لم يسافر جون في عطلته؟</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>لأنه قرّر استثمار أمواله بدلاً من السفر</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>لأن جائحة مفاجئة تسبّبت في إلغاء جميع الرحلات الجوية</t>
+          <t>كيف يمكن تحقيق ربح من تغيّر أسعار الصرف؟</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>بتحويل أموالك إلى عملة ترتفع قيمتها لاحقاً، ثم إعادة التحويل بسعر أفضل</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>بالتحويل ثم إعادة التحويل فوراً بالسعر نفسه</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>لأن مكتب الصرافة رفض تحويل أمواله</t>
+          <t>بالاحتفاظ بأموالك في عملتك المحلية دائماً</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>لأنه خسر أمواله في صفقة تداول</t>
+          <t>بتحويل أموالك إلى عملة تنخفض قيمتها لاحقاً، ثم إعادة التحويل</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>ب</t>
+          <t>أ</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>لأن جائحة مفاجئة تسبّبت في إلغاء جميع الرحلات الجوية</t>
+          <t>بتحويل أموالك إلى عملة ترتفع قيمتها لاحقاً، ثم إعادة التحويل بسعر أفضل</t>
         </is>
       </c>
     </row>
@@ -837,37 +837,37 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>كم دولاراً أسترالياً استلم جون عندما أعاد تحويل دولاراته الأمريكية؟</t>
+          <t>إذا كان الدولار الأسترالي الواحد يساوي 0.70 دولار أمريكي، فكم دولاراً أمريكياً تحصل عليه مقابل 2,000 دولار أسترالي؟</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>700 دولار أسترالي</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>1,000 دولار أسترالي</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>1,100 دولار أسترالي</t>
+          <t>600 دولار أمريكي</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>1,400 دولار أمريكي</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>2,000 دولار أمريكي</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>1,400 دولار أسترالي</t>
+          <t>نحو 2,857 دولاراً أمريكياً</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>ج</t>
+          <t>ب</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>1,100 دولار أسترالي</t>
+          <t>1,400 دولار أمريكي</t>
         </is>
       </c>
     </row>
@@ -892,37 +892,37 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>لماذا حصل جون على مبلغ أكبر مما كان يتوقعه؟</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>لأن قيمة الدولار الأمريكي ارتفعت مقابل الدولار الأسترالي منذ التحويل الأول</t>
+          <t>حوّلت 3,000 يورو إلى دولارات أمريكية عندما كان اليورو الواحد يساوي 1.10 دولار، ثم أعدت تحويل كل الدولارات إلى يورو عندما أصبح اليورو الواحد يساوي 1.00 دولار. كم يورو تحصل عليه؟</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>نحو 2,727 يورو</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>لأنه حصل على تعويض بسبب إلغاء رحلته</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>لأن قيمة الدولار الأمريكي انخفضت مقابل الدولار الأسترالي</t>
+          <t>3,000 يورو</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>3,300 يورو</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>لأن الصرّاف ارتكب خطأً في الحسابات</t>
+          <t>3,630 يورو</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>أ</t>
+          <t>ج</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>لأن قيمة الدولار الأمريكي ارتفعت مقابل الدولار الأسترالي منذ التحويل الأول</t>
+          <t>3,300 يورو</t>
         </is>
       </c>
     </row>
@@ -947,37 +947,37 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>ما مقدار الربح الذي حققه جون من تغيّر سعر الصرف؟</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>100 دولار أمريكي</t>
+          <t>حوّلت 2,000 دولار أسترالي إلى دولارات أمريكية عندما كان الدولار الأسترالي الواحد يساوي 0.75 دولار أمريكي، ثم أعدت تحويل كل الدولارات الأمريكية عندما أصبح يساوي 0.60 دولار أمريكي. كم ربحت أو خسرت بالدولار الأسترالي مقارنةً بمبلغك الأصلي؟</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>ربح 500 دولار أسترالي</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>400 دولار أسترالي</t>
+          <t>ربح 300 دولار أسترالي</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>لم يحقق أي ربح</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>100 دولار أسترالي</t>
+          <t>خسارة 500 دولار أسترالي</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>خسارة 300 دولار أسترالي</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>د</t>
+          <t>أ</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>100 دولار أسترالي</t>
+          <t>ربح 500 دولار أسترالي</t>
         </is>
       </c>
     </row>
@@ -1002,37 +1002,37 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>إذا انخفضت قيمة الدولار الأمريكي مقابل الدولار الأسترالي بين التحويلين، فماذا يحدث عند إعادة التحويل؟</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>سيحصل جون على أقل من 1,000 دولار أسترالي</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>سيحصل جون على 1,100 دولار أسترالي</t>
+          <t>حوّلت 1,000 جنيه إسترليني إلى دولارات أمريكية عندما كان الجنيه يساوي 1.25 دولار، ثم أعدت التحويل عندما أصبح الجنيه يساوي 1.30 دولار. كم جنيهاً تحصل عليه تقريباً؟</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>نحو 950 جنيهاً</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>نحو 962 جنيهاً</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>لن يتمكن جون من إعادة التحويل</t>
+          <t>1,000 جنيه</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>سيحصل جون على 1,000 دولار أسترالي بالضبط</t>
+          <t>1,040 جنيهاً</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>أ</t>
+          <t>ب</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>سيحصل جون على أقل من 1,000 دولار أسترالي</t>
+          <t>نحو 962 جنيهاً</t>
         </is>
       </c>
     </row>
@@ -1062,32 +1062,32 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>الأرباح تأتي من السفر وتحويل العملات فقط</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>الأمر ليس بهذه البساطة، ويجب إكمال المنهاج التعليمي بالكامل</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>لا حاجة إلى التعلّم لأن السوق سهل</t>
+          <t>الأفضل البدء بمبلغ كبير لتعويض أي خسارة</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>الأرباح سهلة لأن الأسعار تتغير باستمرار</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>الأمر ليس بهذه البساطة، ويجب إكمال المنهاج التعليمي بالكامل قبل التداول</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>يكفي فتح حساب حقيقي والبدء فوراً</t>
+          <t>يكفي متابعة أسعار الصرف يومياً لتحقيق الأرباح</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>ب</t>
+          <t>ج</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>الأمر ليس بهذه البساطة، ويجب إكمال المنهاج التعليمي بالكامل</t>
+          <t>الأمر ليس بهذه البساطة، ويجب إكمال المنهاج التعليمي بالكامل قبل التداول</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Quiz bank: general lesson 2 and 3 questions (no story character)
At the client's request, the four questions in lessons 2 and 3 that named
the story character now ask about forex in general. Lesson 3 gains a
worked pair-quote problem (GBP/USD) with typical-mistake options.
PDF and Excel rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C9b7SosS81gsG93Ye2rtJ2
</commit_message>
<xml_diff>
--- a/axi-academy/quizzes/AxiAcademy_QuestionBank.xlsx
+++ b/axi-academy/quizzes/AxiAcademy_QuestionBank.xlsx
@@ -1442,7 +1442,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>ما فائدة ساعات عمل سوق الفوركس الطويلة لمتداول مثل جون؟</t>
+          <t>ما فائدة ساعات عمل سوق الفوركس الطويلة للمتداول؟</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1672,22 +1672,22 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
+          <t>على سعر الذهب مقابل الفضة</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
           <t>على أسعار الفائدة فقط</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>على تقلبات سعر الصرف بين عملتين</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>على سعر الذهب مقابل الفضة</t>
-        </is>
-      </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>ج</t>
+          <t>د</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1772,37 +1772,37 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>لماذا كان زوج AUD/USD هو الزوج المعني في مثال جون؟</t>
+          <t>إذا كان سعر زوج GBP/USD يساوي 1.2500، فكم دولاراً أمريكياً تحتاج لشراء 1,000 جنيه إسترليني؟</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>لأن الوسيط لا يعرض أي زوج غيره</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>لأنه أراد تحويل دولاراته الأسترالية إلى دولارات أمريكية للسفر إلى أمريكا</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>لأنه أكثر أزواج العملات تداولاً في العالم</t>
+          <t>800 دولار</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>1,000 دولار</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>1,250 دولاراً</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>لأن الدولار الأسترالي يساوي الدولار الأمريكي دائماً</t>
+          <t>12,500 دولار</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>ب</t>
+          <t>ج</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>لأنه أراد تحويل دولاراته الأسترالية إلى دولارات أمريكية للسفر إلى أمريكا</t>
+          <t>1,250 دولاراً</t>
         </is>
       </c>
     </row>
@@ -1832,27 +1832,27 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
+          <t>العملتان متساويتان في القيمة</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>الدولار الأسترالي الواحد يساوي 0.7000 دولار أمريكي</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>الدولار الأمريكي الواحد يساوي 0.7000 دولار أسترالي</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
           <t>الدولار الأسترالي الواحد يساوي 7 دولارات أمريكية</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>الدولار الأمريكي الواحد يساوي 0.7000 دولار أسترالي</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>العملتان متساويتان في القيمة</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>الدولار الأسترالي الواحد يساوي 0.7000 دولار أمريكي</t>
-        </is>
-      </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>د</t>
+          <t>ب</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -1882,32 +1882,32 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>ما الخياران اللذان لاحظهما جون على منصة التداول؟</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
+          <t>ما الخياران الأساسيان اللذان تجدهما على منصة التداول لفتح صفقة؟</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>جني الأرباح ووقف الخسارة</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>الإيداع والسحب</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>الشراء والبيع</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>الافتتاح والإغلاق</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>الإيداع والسحب</t>
-        </is>
-      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>الربح والخسارة</t>
+          <t>الرافعة المالية والهامش</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>أ</t>
+          <t>ج</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -1937,37 +1937,37 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>متى يشتري جون زوج AUD/USD؟</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>عندما تتساوى قيمة العملتين</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>عندما يتوقع أن ترتفع قيمة الزوج</t>
+          <t>متى تشتري زوج AUD/USD؟</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>عندما تتوقع أن ترتفع قيمة الزوج</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>عندما تتوقع أن يقوى الدولار الأمريكي أمام الدولار الأسترالي</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>عندما يكون السوق مغلقاً</t>
+          <t>عندما تتوقع أن تنخفض قيمة الزوج</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>عندما يتوقع أن تنخفض قيمة الزوج</t>
+          <t>عندما يكون سعر الزوج أقل من 1.0000</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>ب</t>
+          <t>أ</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>عندما يتوقع أن ترتفع قيمة الزوج</t>
+          <t>عندما تتوقع أن ترتفع قيمة الزوج</t>
         </is>
       </c>
     </row>
@@ -2000,16 +2000,16 @@
           <t>عندما يُغلق السوق في نهاية الأسبوع</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>عندما يقوى الدولار الأسترالي أمام الدولار الأمريكي، أو يضعف الدولار الأمريكي أمامه</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>عندما تضعف العملتان معاً بالقدر نفسه</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>عندما يقوى الدولار الأسترالي أمام الدولار الأمريكي، أو يضعف الدولار الأمريكي أمامه</t>
-        </is>
-      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>عندما يقوى الدولار الأمريكي أمام الدولار الأسترالي</t>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>ج</t>
+          <t>ب</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2052,17 +2052,17 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
+          <t>في بداية كل أسبوع</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>عند تحقيق أي ربح</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
           <t>عندما تتوقع أن ترتفع قيمة الزوج</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>في بداية كل أسبوع</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>عند تحقيق أي ربح</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
+          <t>يرتفع</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>ينخفض</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
           <t>يتضاعف</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>يرتفع</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>ينخفض</t>
-        </is>
-      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
           <t>يبقى ثابتاً</t>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>ج</t>
+          <t>ب</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2160,29 +2160,29 @@
           <t>ارتفع سعر AUD/USD من 0.7000 إلى 0.7100. أي صفقة كانت ستربح؟</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>لا صفقة منهما</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>صفقة البيع</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>الصفقتان معاً</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>صفقة الشراء</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>صفقة البيع</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>لا صفقة منهما</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>الصفقتان معاً</t>
-        </is>
-      </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>أ</t>
+          <t>د</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">

</xml_diff>